<commit_message>
Auto-actualizacion de sorteos en vivo
</commit_message>
<xml_diff>
--- a/Loteria ag/Recientes.xlsx
+++ b/Loteria ag/Recientes.xlsx
@@ -464,13 +464,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="C2" t="n">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="D2" t="n">
-        <v>57</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">

</xml_diff>